<commit_message>
feat: update the ETL
</commit_message>
<xml_diff>
--- a/data/processed/2024-03/MIR_2024-03_diario.xlsx
+++ b/data/processed/2024-03/MIR_2024-03_diario.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="90">
   <si>
     <t>FECHA</t>
   </si>
@@ -218,6 +218,9 @@
     <t>Fuente</t>
   </si>
   <si>
+    <t>Proceso</t>
+  </si>
+  <si>
     <t>Norma</t>
   </si>
   <si>
@@ -246,6 +249,9 @@
   </si>
   <si>
     <t>SEMADET Jalisco, BD_2024.xlsx (hoja Data), estación Miravalle (MIR). Unidades de la hoja Param.</t>
+  </si>
+  <si>
+    <t>etl.py (limpieza del año) → calculos.py (Archivo1 horario y Archivo2 diario) → procesar.py (JSON del sitio y Excel).</t>
   </si>
   <si>
     <t>NOM-172-SEMARNAT-2023. Criterios validados en Actividades 5 y 6 (SFE, enero 2025).</t>
@@ -4117,7 +4123,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="61" width="14.7109375" customWidth="1"/>
@@ -4136,7 +4142,7 @@
         <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -4144,7 +4150,7 @@
         <v>67</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -4152,31 +4158,31 @@
         <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -4184,7 +4190,7 @@
         <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -4192,7 +4198,7 @@
         <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -4200,7 +4206,7 @@
         <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4208,7 +4214,7 @@
         <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -4216,7 +4222,7 @@
         <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -4224,7 +4230,15 @@
         <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Nuevo diseño visual, agregando visuales informativos y apegados a la NOM
</commit_message>
<xml_diff>
--- a/data/processed/2024-03/MIR_2024-03_diario.xlsx
+++ b/data/processed/2024-03/MIR_2024-03_diario.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="94">
   <si>
     <t>FECHA</t>
   </si>
@@ -233,6 +233,12 @@
     <t>Bandas</t>
   </si>
   <si>
+    <t>Redondeo</t>
+  </si>
+  <si>
+    <t>Mensajes</t>
+  </si>
+  <si>
     <t>Suficiencia diaria</t>
   </si>
   <si>
@@ -269,7 +275,13 @@
     <t>NowCast 12 h con la función de referencia de la profesora (≥ 2 de las 3 horas recientes; W ≥ 0.5; factor 0.714 PM10 / 0.694 PM2.5). Diario = promedio 24 h redondeado a entero.</t>
   </si>
   <si>
-    <t>O3: 0.058/0.090/0.135/0.175 ppm · CO: 5/9/12/16 ppm · PM10: 45/60/132/213 µg/m³ · PM2.5: 15/33/79/130 µg/m³.</t>
+    <t>Tablas 4 a 9 de la NOM. O3: 0.058/0.090/0.135/0.175 ppm · CO: 5/9/12/16 ppm · PM10: 45/60/132/213 µg/m³ · PM2.5: 15/33/79/130 µg/m³. Para partículas se usa la columna «a partir de enero de 2024», que corresponde al año de los datos.</t>
+  </si>
+  <si>
+    <t>Numeral 5.2.4: O3 a 3 decimales, CO a 2 y PM a entero; si la cifra siguiente es 5 o más, se sube. En marzo 2024 el redondeo interno de la función NowCast de referencia coincide con esta regla en todas las horas.</t>
+  </si>
+  <si>
+    <t>Tabla 12 de la NOM, textos oficiales para tres grupos: población en general; menores de 12 años y personas gestantes; personas con enfermedades cardiovasculares o respiratorias y mayores de 60 años.</t>
   </si>
   <si>
     <t>≥ 18 de 24 datos horarios válidos (75 %) por contaminante; si no cumple, no se calcula indicador.</t>
@@ -1847,7 +1859,7 @@
         <v>46</v>
       </c>
       <c r="F12">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G12" t="s">
         <v>48</v>
@@ -2281,7 +2293,7 @@
         <v>46</v>
       </c>
       <c r="F16">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G16" t="s">
         <v>48</v>
@@ -3458,7 +3470,7 @@
         <v>46</v>
       </c>
       <c r="J27">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K27" t="s">
         <v>50</v>
@@ -4123,7 +4135,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="61" width="14.7109375" customWidth="1"/>
@@ -4142,7 +4154,7 @@
         <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -4150,7 +4162,7 @@
         <v>67</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -4158,7 +4170,7 @@
         <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -4166,7 +4178,7 @@
         <v>69</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -4174,7 +4186,7 @@
         <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -4182,7 +4194,7 @@
         <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -4190,7 +4202,7 @@
         <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -4198,7 +4210,7 @@
         <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -4206,7 +4218,7 @@
         <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -4214,7 +4226,7 @@
         <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -4222,7 +4234,7 @@
         <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -4230,7 +4242,7 @@
         <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -4238,7 +4250,23 @@
         <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>89</v>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>